<commit_message>
Grok Pass 3: apply global canonical marquees + deploy
Apply handoff/global-marquee-pass2/CANONICAL-MARQUEES.json to 20 commercial
partners (direct route_id bind, no re-stamp). Finance cascade, inheritance
gates, journey scrub, and production deploy to navier-atlas.vercel.app.

- apply_canonical_marquees_global.py + run_global_inheritance_pass3.sh
- validate_partner_inheritance: skip intentional_null phases
- Post-reseal journey scrub + Thailand/Caribbean fidelity fixes
</commit_message>
<xml_diff>
--- a/finance/_refresh_airasia-move.xlsx
+++ b/finance/_refresh_airasia-move.xlsx
@@ -11759,11 +11759,11 @@
         </is>
       </c>
       <c r="C11" s="39" t="n">
-        <v>0.1101</v>
+        <v>0.1</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>New-entrant ~11% share of today's pool (= the published floor).</t>
+          <t>New-entrant ~10% share of today's pool (= the published floor).</t>
         </is>
       </c>
     </row>
@@ -11836,7 +11836,7 @@
     <row r="18">
       <c r="A18" s="25" t="inlineStr">
         <is>
-          <t>SOM full network (~11% capture, today, +greenfield)</t>
+          <t>SOM full network (~10% capture, today, +greenfield)</t>
         </is>
       </c>
       <c r="B18" s="50">
@@ -11853,7 +11853,7 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Floor posture (~11% captive capture, today's demand) extended across the whole mapped network.</t>
+          <t>Floor posture (~10% captive capture, today's demand) extended across the whole mapped network.</t>
         </is>
       </c>
     </row>

</xml_diff>